<commit_message>
Add Aasted detachment hooks and demoulding subphases
</commit_message>
<xml_diff>
--- a/outputs/aasted3_run_comparison/summary/aasted3_contour_data.xlsx
+++ b/outputs/aasted3_run_comparison/summary/aasted3_contour_data.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hotspot Delta Matrix" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contour Data'!$A$1:$N$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hotspot Delta Matrix'!$A$1:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contour Data'!$A$1:$N$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hotspot Delta Matrix'!$A$1:$G$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -437,7 +437,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
@@ -1056,140 +1056,140 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>demoulding</t>
+          <t>demoulding_twisting</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>1792</v>
       </c>
       <c r="D13" t="n">
-        <v>1869</v>
+        <v>1799</v>
       </c>
       <c r="E13" t="n">
-        <v>77</v>
+        <v>7</v>
       </c>
       <c r="F13" t="n">
-        <v>63.09195201417348</v>
+        <v>61.94264913739641</v>
       </c>
       <c r="G13" t="n">
-        <v>15.28274197048611</v>
+        <v>15.13020833333333</v>
       </c>
       <c r="H13" t="n">
-        <v>14.17510308159722</v>
+        <v>13.97721354166667</v>
       </c>
       <c r="I13" t="n">
-        <v>14.03700086805556</v>
+        <v>13.87109375</v>
       </c>
       <c r="J13" t="n">
-        <v>13.92442491319444</v>
+        <v>13.67447916666667</v>
       </c>
       <c r="K13" t="n">
-        <v>14.08390299479167</v>
+        <v>13.4892578125</v>
       </c>
       <c r="L13" t="n">
-        <v>14.57793511284722</v>
+        <v>14.39908854166667</v>
       </c>
       <c r="M13" t="n">
-        <v>15.08837890625</v>
+        <v>14.63248697916667</v>
       </c>
       <c r="N13" t="n">
-        <v>14.14567057291667</v>
+        <v>13.67740885416667</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>reference_2291-4160</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>movement_to_conditioning</t>
+          <t>demoulding_vibration</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1799</v>
       </c>
       <c r="D14" t="n">
-        <v>67</v>
+        <v>1860</v>
       </c>
       <c r="E14" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F14" t="n">
-        <v>30.41959307787037</v>
+        <v>63.05714789807157</v>
       </c>
       <c r="G14" t="n">
-        <v>22.12476325757576</v>
+        <v>15.27720905172414</v>
       </c>
       <c r="H14" t="n">
-        <v>22.38299005681818</v>
+        <v>14.1669921875</v>
       </c>
       <c r="I14" t="n">
-        <v>21.84537760416667</v>
+        <v>14.02693965517241</v>
       </c>
       <c r="J14" t="n">
-        <v>22.62479285037879</v>
+        <v>13.91594827586207</v>
       </c>
       <c r="K14" t="n">
-        <v>21.78666548295455</v>
+        <v>14.08637526939655</v>
       </c>
       <c r="L14" t="n">
-        <v>22.20513731060606</v>
+        <v>14.56805630387931</v>
       </c>
       <c r="M14" t="n">
-        <v>22.33262310606061</v>
+        <v>15.07980872844828</v>
       </c>
       <c r="N14" t="n">
-        <v>21.66850142045455</v>
+        <v>14.13520339439655</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>reference_2291-4160</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>mould_conditioning</t>
+          <t>final_demoulding</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>67</v>
+        <v>1860</v>
       </c>
       <c r="D15" t="n">
-        <v>493</v>
+        <v>1869</v>
       </c>
       <c r="E15" t="n">
-        <v>426</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
-        <v>27.64735353773485</v>
+        <v>64.20625901349527</v>
       </c>
       <c r="G15" t="n">
-        <v>22.32362272593897</v>
+        <v>15.437255859375</v>
       </c>
       <c r="H15" t="n">
-        <v>22.73446669600939</v>
+        <v>14.38232421875</v>
       </c>
       <c r="I15" t="n">
-        <v>22.15354955252348</v>
+        <v>14.234375</v>
       </c>
       <c r="J15" t="n">
-        <v>22.69943423562206</v>
+        <v>14.17333984375</v>
       </c>
       <c r="K15" t="n">
-        <v>22.3557851012324</v>
+        <v>14.511962890625</v>
       </c>
       <c r="L15" t="n">
-        <v>22.33242095803991</v>
+        <v>14.78369140625</v>
       </c>
       <c r="M15" t="n">
-        <v>23.21314278902582</v>
+        <v>15.492431640625</v>
       </c>
       <c r="N15" t="n">
-        <v>22.36638057511737</v>
+        <v>14.57275390625</v>
       </c>
     </row>
     <row r="16">
@@ -1200,44 +1200,44 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>deposition_transfer</t>
+          <t>movement_to_conditioning</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>493</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>600</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="F16" t="n">
-        <v>18.40996017253675</v>
+        <v>30.41959307787037</v>
       </c>
       <c r="G16" t="n">
-        <v>27.84138093171296</v>
+        <v>22.12476325757576</v>
       </c>
       <c r="H16" t="n">
-        <v>28.89122178819444</v>
+        <v>22.38299005681818</v>
       </c>
       <c r="I16" t="n">
-        <v>28.3255931712963</v>
+        <v>21.84537760416667</v>
       </c>
       <c r="J16" t="n">
-        <v>28.19858579282407</v>
+        <v>22.62479285037879</v>
       </c>
       <c r="K16" t="n">
-        <v>28.04537398726852</v>
+        <v>21.78666548295455</v>
       </c>
       <c r="L16" t="n">
-        <v>27.98318142361111</v>
+        <v>22.20513731060606</v>
       </c>
       <c r="M16" t="n">
-        <v>28.87076822916667</v>
+        <v>22.33262310606061</v>
       </c>
       <c r="N16" t="n">
-        <v>27.83769169560185</v>
+        <v>21.66850142045455</v>
       </c>
     </row>
     <row r="17">
@@ -1248,44 +1248,44 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>vibration_warming</t>
+          <t>mould_conditioning</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>600</v>
+        <v>67</v>
       </c>
       <c r="D17" t="n">
-        <v>646</v>
+        <v>493</v>
       </c>
       <c r="E17" t="n">
-        <v>46</v>
+        <v>426</v>
       </c>
       <c r="F17" t="n">
-        <v>20.08367390689834</v>
+        <v>27.64735353773485</v>
       </c>
       <c r="G17" t="n">
-        <v>28.08763586956522</v>
+        <v>22.32362272593897</v>
       </c>
       <c r="H17" t="n">
-        <v>28.41015625</v>
+        <v>22.73446669600939</v>
       </c>
       <c r="I17" t="n">
-        <v>28.33793308423913</v>
+        <v>22.15354955252348</v>
       </c>
       <c r="J17" t="n">
-        <v>27.99660326086957</v>
+        <v>22.69943423562206</v>
       </c>
       <c r="K17" t="n">
-        <v>27.96586277173913</v>
+        <v>22.3557851012324</v>
       </c>
       <c r="L17" t="n">
-        <v>28.1410495923913</v>
+        <v>22.33242095803991</v>
       </c>
       <c r="M17" t="n">
-        <v>27.27381963315218</v>
+        <v>23.21314278902582</v>
       </c>
       <c r="N17" t="n">
-        <v>27.521484375</v>
+        <v>22.36638057511737</v>
       </c>
     </row>
     <row r="18">
@@ -1296,44 +1296,44 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>transition_to_cooling</t>
+          <t>deposition_transfer</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>646</v>
+        <v>493</v>
       </c>
       <c r="D18" t="n">
-        <v>794</v>
+        <v>600</v>
       </c>
       <c r="E18" t="n">
-        <v>148</v>
+        <v>107</v>
       </c>
       <c r="F18" t="n">
-        <v>22.5690515473382</v>
+        <v>18.40996017253675</v>
       </c>
       <c r="G18" t="n">
-        <v>27.60821322737069</v>
+        <v>27.84138093171296</v>
       </c>
       <c r="H18" t="n">
-        <v>27.67869410021552</v>
+        <v>28.89122178819444</v>
       </c>
       <c r="I18" t="n">
-        <v>27.77015422952586</v>
+        <v>28.3255931712963</v>
       </c>
       <c r="J18" t="n">
-        <v>27.29754849137931</v>
+        <v>28.19858579282407</v>
       </c>
       <c r="K18" t="n">
-        <v>27.37843480603448</v>
+        <v>28.04537398726852</v>
       </c>
       <c r="L18" t="n">
-        <v>27.43121969288793</v>
+        <v>27.98318142361111</v>
       </c>
       <c r="M18" t="n">
-        <v>24.94090113146552</v>
+        <v>28.87076822916667</v>
       </c>
       <c r="N18" t="n">
-        <v>26.74345029633621</v>
+        <v>27.83769169560185</v>
       </c>
     </row>
     <row r="19">
@@ -1344,44 +1344,44 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>cooling_1</t>
+          <t>vibration_warming</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>794</v>
+        <v>600</v>
       </c>
       <c r="D19" t="n">
-        <v>891</v>
+        <v>646</v>
       </c>
       <c r="E19" t="n">
-        <v>97</v>
+        <v>46</v>
       </c>
       <c r="F19" t="n">
-        <v>31.26008628754608</v>
+        <v>20.08367390689834</v>
       </c>
       <c r="G19" t="n">
-        <v>26.036865234375</v>
+        <v>28.08763586956522</v>
       </c>
       <c r="H19" t="n">
-        <v>25.24886067708333</v>
+        <v>28.41015625</v>
       </c>
       <c r="I19" t="n">
-        <v>25.42427571614583</v>
+        <v>28.33793308423913</v>
       </c>
       <c r="J19" t="n">
-        <v>25.34897867838542</v>
+        <v>27.99660326086957</v>
       </c>
       <c r="K19" t="n">
-        <v>24.54620361328125</v>
+        <v>27.96586277173913</v>
       </c>
       <c r="L19" t="n">
-        <v>25.5823974609375</v>
+        <v>28.1410495923913</v>
       </c>
       <c r="M19" t="n">
-        <v>19.31650797526042</v>
+        <v>27.27381963315218</v>
       </c>
       <c r="N19" t="n">
-        <v>23.711181640625</v>
+        <v>27.521484375</v>
       </c>
     </row>
     <row r="20">
@@ -1392,44 +1392,44 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>cooling_2</t>
+          <t>transition_to_cooling</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>891</v>
+        <v>646</v>
       </c>
       <c r="D20" t="n">
-        <v>1040</v>
+        <v>794</v>
       </c>
       <c r="E20" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F20" t="n">
-        <v>43.80239717798488</v>
+        <v>22.5690515473382</v>
       </c>
       <c r="G20" t="n">
-        <v>22.29559491131757</v>
+        <v>27.60821322737069</v>
       </c>
       <c r="H20" t="n">
-        <v>21.28576330236486</v>
+        <v>27.67869410021552</v>
       </c>
       <c r="I20" t="n">
-        <v>20.90987911739865</v>
+        <v>27.77015422952586</v>
       </c>
       <c r="J20" t="n">
-        <v>22.23527238175676</v>
+        <v>27.29754849137931</v>
       </c>
       <c r="K20" t="n">
-        <v>19.58548880912162</v>
+        <v>27.37843480603448</v>
       </c>
       <c r="L20" t="n">
-        <v>21.83449904983108</v>
+        <v>27.43121969288793</v>
       </c>
       <c r="M20" t="n">
-        <v>14.56046769425676</v>
+        <v>24.94090113146552</v>
       </c>
       <c r="N20" t="n">
-        <v>19.36277977195946</v>
+        <v>26.74345029633621</v>
       </c>
     </row>
     <row r="21">
@@ -1440,44 +1440,44 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>cooling_3</t>
+          <t>cooling_1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1040</v>
+        <v>794</v>
       </c>
       <c r="D21" t="n">
-        <v>1152</v>
+        <v>891</v>
       </c>
       <c r="E21" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="F21" t="n">
-        <v>46.59697963747105</v>
+        <v>31.26008628754608</v>
       </c>
       <c r="G21" t="n">
-        <v>19.89169034090909</v>
+        <v>26.036865234375</v>
       </c>
       <c r="H21" t="n">
-        <v>18.7251953125</v>
+        <v>25.24886067708333</v>
       </c>
       <c r="I21" t="n">
-        <v>18.09115767045455</v>
+        <v>25.42427571614583</v>
       </c>
       <c r="J21" t="n">
-        <v>20.30078125</v>
+        <v>25.34897867838542</v>
       </c>
       <c r="K21" t="n">
-        <v>17.33510298295455</v>
+        <v>24.54620361328125</v>
       </c>
       <c r="L21" t="n">
-        <v>19.80079900568182</v>
+        <v>25.5823974609375</v>
       </c>
       <c r="M21" t="n">
-        <v>14.14669744318182</v>
+        <v>19.31650797526042</v>
       </c>
       <c r="N21" t="n">
-        <v>17.10118963068182</v>
+        <v>23.711181640625</v>
       </c>
     </row>
     <row r="22">
@@ -1488,44 +1488,44 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>cooling_4</t>
+          <t>cooling_2</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1152</v>
+        <v>891</v>
       </c>
       <c r="D22" t="n">
-        <v>1307</v>
+        <v>1040</v>
       </c>
       <c r="E22" t="n">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F22" t="n">
-        <v>49.02330759342392</v>
+        <v>43.80239717798488</v>
       </c>
       <c r="G22" t="n">
-        <v>19.14593184621711</v>
+        <v>22.29559491131757</v>
       </c>
       <c r="H22" t="n">
-        <v>17.85641961348684</v>
+        <v>21.28576330236486</v>
       </c>
       <c r="I22" t="n">
-        <v>17.23269171463816</v>
+        <v>20.90987911739865</v>
       </c>
       <c r="J22" t="n">
-        <v>19.48482473273026</v>
+        <v>22.23527238175676</v>
       </c>
       <c r="K22" t="n">
-        <v>16.58528217516447</v>
+        <v>19.58548880912162</v>
       </c>
       <c r="L22" t="n">
-        <v>19.27977230674342</v>
+        <v>21.83449904983108</v>
       </c>
       <c r="M22" t="n">
-        <v>13.66275185032895</v>
+        <v>14.56046769425676</v>
       </c>
       <c r="N22" t="n">
-        <v>16.06689453125</v>
+        <v>19.36277977195946</v>
       </c>
     </row>
     <row r="23">
@@ -1536,44 +1536,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>less_periodic_cooling_2</t>
+          <t>cooling_3</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1307</v>
+        <v>1040</v>
       </c>
       <c r="D23" t="n">
-        <v>2035</v>
+        <v>1152</v>
       </c>
       <c r="E23" t="n">
-        <v>728</v>
+        <v>112</v>
       </c>
       <c r="F23" t="n">
-        <v>49.96856924279216</v>
+        <v>46.59697963747105</v>
       </c>
       <c r="G23" t="n">
-        <v>16.77396771121884</v>
+        <v>19.89169034090909</v>
       </c>
       <c r="H23" t="n">
-        <v>14.41952692174515</v>
+        <v>18.7251953125</v>
       </c>
       <c r="I23" t="n">
-        <v>14.14381979310942</v>
+        <v>18.09115767045455</v>
       </c>
       <c r="J23" t="n">
-        <v>15.66035102146814</v>
+        <v>20.30078125</v>
       </c>
       <c r="K23" t="n">
-        <v>14.12902798216759</v>
+        <v>17.33510298295455</v>
       </c>
       <c r="L23" t="n">
-        <v>16.64899746797091</v>
+        <v>19.80079900568182</v>
       </c>
       <c r="M23" t="n">
-        <v>12.36247781769391</v>
+        <v>14.14669744318182</v>
       </c>
       <c r="N23" t="n">
-        <v>13.34616570723684</v>
+        <v>17.10118963068182</v>
       </c>
     </row>
     <row r="24">
@@ -1584,44 +1584,44 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>transition_2</t>
+          <t>cooling_4</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2035</v>
+        <v>1152</v>
       </c>
       <c r="D24" t="n">
-        <v>2074</v>
+        <v>1307</v>
       </c>
       <c r="E24" t="n">
-        <v>39</v>
+        <v>155</v>
       </c>
       <c r="F24" t="n">
-        <v>47.81232937856691</v>
+        <v>49.02330759342392</v>
       </c>
       <c r="G24" t="n">
-        <v>15.203125</v>
+        <v>19.14593184621711</v>
       </c>
       <c r="H24" t="n">
-        <v>13.226953125</v>
+        <v>17.85641961348684</v>
       </c>
       <c r="I24" t="n">
-        <v>13.240234375</v>
+        <v>17.23269171463816</v>
       </c>
       <c r="J24" t="n">
-        <v>13.610302734375</v>
+        <v>19.48482473273026</v>
       </c>
       <c r="K24" t="n">
-        <v>13.287548828125</v>
+        <v>16.58528217516447</v>
       </c>
       <c r="L24" t="n">
-        <v>14.919091796875</v>
+        <v>19.27977230674342</v>
       </c>
       <c r="M24" t="n">
-        <v>13.68056640625</v>
+        <v>13.66275185032895</v>
       </c>
       <c r="N24" t="n">
-        <v>12.71396484375</v>
+        <v>16.06689453125</v>
       </c>
     </row>
     <row r="25">
@@ -1632,48 +1632,240 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>demoulding</t>
+          <t>less_periodic_cooling_2</t>
         </is>
       </c>
       <c r="C25" t="n">
+        <v>1307</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2035</v>
+      </c>
+      <c r="E25" t="n">
+        <v>728</v>
+      </c>
+      <c r="F25" t="n">
+        <v>49.96856924279216</v>
+      </c>
+      <c r="G25" t="n">
+        <v>16.77396771121884</v>
+      </c>
+      <c r="H25" t="n">
+        <v>14.41952692174515</v>
+      </c>
+      <c r="I25" t="n">
+        <v>14.14381979310942</v>
+      </c>
+      <c r="J25" t="n">
+        <v>15.66035102146814</v>
+      </c>
+      <c r="K25" t="n">
+        <v>14.12902798216759</v>
+      </c>
+      <c r="L25" t="n">
+        <v>16.64899746797091</v>
+      </c>
+      <c r="M25" t="n">
+        <v>12.36247781769391</v>
+      </c>
+      <c r="N25" t="n">
+        <v>13.34616570723684</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>old-configuration</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>transition_2</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2035</v>
+      </c>
+      <c r="D26" t="n">
         <v>2074</v>
       </c>
-      <c r="D25" t="n">
+      <c r="E26" t="n">
+        <v>39</v>
+      </c>
+      <c r="F26" t="n">
+        <v>47.81232937856691</v>
+      </c>
+      <c r="G26" t="n">
+        <v>15.203125</v>
+      </c>
+      <c r="H26" t="n">
+        <v>13.226953125</v>
+      </c>
+      <c r="I26" t="n">
+        <v>13.240234375</v>
+      </c>
+      <c r="J26" t="n">
+        <v>13.610302734375</v>
+      </c>
+      <c r="K26" t="n">
+        <v>13.287548828125</v>
+      </c>
+      <c r="L26" t="n">
+        <v>14.919091796875</v>
+      </c>
+      <c r="M26" t="n">
+        <v>13.68056640625</v>
+      </c>
+      <c r="N26" t="n">
+        <v>12.71396484375</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>old-configuration</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>demoulding_twisting</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2074</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2081</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" t="n">
+        <v>45.34554205390111</v>
+      </c>
+      <c r="G27" t="n">
+        <v>15.365234375</v>
+      </c>
+      <c r="H27" t="n">
+        <v>13.4091796875</v>
+      </c>
+      <c r="I27" t="n">
+        <v>13.37890625</v>
+      </c>
+      <c r="J27" t="n">
+        <v>13.83072916666667</v>
+      </c>
+      <c r="K27" t="n">
+        <v>13.61165364583333</v>
+      </c>
+      <c r="L27" t="n">
+        <v>15.05859375</v>
+      </c>
+      <c r="M27" t="n">
+        <v>14.35286458333333</v>
+      </c>
+      <c r="N27" t="n">
+        <v>13.24251302083333</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>old-configuration</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>demoulding_vibration</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2081</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2137</v>
+      </c>
+      <c r="E28" t="n">
+        <v>56</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-4.087239910377834</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2.28443287037037</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.99609375</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.990668402777778</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2.058702256944445</v>
+      </c>
+      <c r="K28" t="n">
+        <v>2.03833912037037</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2.237232349537037</v>
+      </c>
+      <c r="M28" t="n">
+        <v>2.177734375</v>
+      </c>
+      <c r="N28" t="n">
+        <v>1.976345486111111</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>old-configuration</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>final_demoulding</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2137</v>
+      </c>
+      <c r="D29" t="n">
         <v>2141</v>
       </c>
-      <c r="E25" t="n">
-        <v>67</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.02128589317193197</v>
-      </c>
-      <c r="G25" t="n">
-        <v>3.36798095703125</v>
-      </c>
-      <c r="H25" t="n">
-        <v>2.941314697265625</v>
-      </c>
-      <c r="I25" t="n">
-        <v>2.93389892578125</v>
-      </c>
-      <c r="J25" t="n">
-        <v>3.033660888671875</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2.995941162109375</v>
-      </c>
-      <c r="L25" t="n">
-        <v>3.299407958984375</v>
-      </c>
-      <c r="M25" t="n">
-        <v>3.18304443359375</v>
-      </c>
-      <c r="N25" t="n">
-        <v>2.909027099609375</v>
+      <c r="E29" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N25"/>
+  <autoFilter ref="A1:N29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1684,7 +1876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1849,23 +2041,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>demoulding</t>
+          <t>demoulding_twisting</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.2527282714843748</v>
+        <v>1.156705729166669</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1739379882812502</v>
+        <v>-0.7993489583333311</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1813537597656252</v>
+        <v>-0.8296223958333311</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.08159179687500018</v>
+        <v>-0.377799479166665</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1841552734374998</v>
+        <v>0.8500651041666689</v>
       </c>
     </row>
     <row r="7">
@@ -1876,23 +2068,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>deposition_transfer</t>
+          <t>demoulding_vibration</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.4066116898148167</v>
+        <v>0.1710069444444442</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6432291666666643</v>
+        <v>-0.117332175925926</v>
       </c>
       <c r="E7" t="n">
-        <v>0.07760054976851904</v>
+        <v>-0.1227575231481484</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.04940682870370594</v>
+        <v>-0.0547236689814814</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.2648111979166679</v>
+        <v>0.1238064236111112</v>
       </c>
     </row>
     <row r="8">
@@ -1903,23 +2095,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>less_periodic_cooling_2</t>
+          <t>deposition_transfer</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.244635128116345</v>
+        <v>-0.4066116898148167</v>
       </c>
       <c r="D8" t="n">
-        <v>-1.10980566135734</v>
+        <v>0.6432291666666643</v>
       </c>
       <c r="E8" t="n">
-        <v>-1.385512789993074</v>
+        <v>0.07760054976851904</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1310184383656505</v>
+        <v>-0.04940682870370594</v>
       </c>
       <c r="G8" t="n">
-        <v>1.119664884868422</v>
+        <v>-0.2648111979166679</v>
       </c>
     </row>
     <row r="9">
@@ -1930,23 +2122,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>mould_conditioning</t>
+          <t>final_demoulding</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.1250761076877893</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.285767862382631</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.2951492811032814</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0.250735401995307</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1162778755868494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1957,23 +2149,23 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>movement_to_conditioning</t>
+          <t>less_periodic_cooling_2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-0.1118489583333364</v>
+        <v>1.244635128116345</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1463778409090892</v>
+        <v>-1.10980566135734</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.3912346117424264</v>
+        <v>-1.385512789993074</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3881806344696948</v>
+        <v>0.1310184383656505</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.03147490530303187</v>
+        <v>1.119664884868422</v>
       </c>
     </row>
     <row r="11">
@@ -1984,23 +2176,23 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>transition_2</t>
+          <t>mould_conditioning</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1.16318359375</v>
+        <v>-0.1250761076877893</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.81298828125</v>
+        <v>0.285767862382631</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.7997070312499996</v>
+        <v>-0.2951492811032814</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.4296386718749989</v>
+        <v>0.250735401995307</v>
       </c>
       <c r="G11" t="n">
-        <v>0.879150390625</v>
+        <v>-0.1162778755868494</v>
       </c>
     </row>
     <row r="12">
@@ -2011,23 +2203,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>transition_to_cooling</t>
+          <t>movement_to_conditioning</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.05104727909483131</v>
+        <v>-0.1118489583333364</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1215281519396569</v>
+        <v>0.1463778409090892</v>
       </c>
       <c r="E12" t="n">
-        <v>0.2129882812500021</v>
+        <v>-0.3912346117424264</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.2596174568965495</v>
+        <v>0.3881806344696948</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1259462553879267</v>
+        <v>-0.03147490530303187</v>
       </c>
     </row>
     <row r="13">
@@ -2038,77 +2230,77 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>vibration_warming</t>
+          <t>transition_2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.1070397418478244</v>
+        <v>1.16318359375</v>
       </c>
       <c r="D13" t="n">
-        <v>0.215480638586957</v>
+        <v>-0.81298828125</v>
       </c>
       <c r="E13" t="n">
-        <v>0.143257472826086</v>
+        <v>-0.7997070312499996</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.1980723505434767</v>
+        <v>-0.4296386718749989</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.05362601902173836</v>
+        <v>0.879150390625</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>reference_2291-4160</t>
+          <t>old-configuration</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>cooling_1</t>
+          <t>transition_to_cooling</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.7528021364795947</v>
+        <v>0.05104727909483131</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.6453364158163239</v>
+        <v>0.1215281519396569</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.4081911670918323</v>
+        <v>0.2129882812500021</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.1532884247448933</v>
+        <v>-0.2596174568965495</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4540138711734727</v>
+        <v>-0.1259462553879267</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>reference_2291-4160</t>
+          <t>old-configuration</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>cooling_2</t>
+          <t>vibration_warming</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.9842759284420275</v>
+        <v>-0.1070397418478244</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.8306442481884062</v>
+        <v>0.215480638586957</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1593636775362341</v>
+        <v>0.143257472826086</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.7778391077898554</v>
+        <v>-0.1980723505434767</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7835711050724647</v>
+        <v>-0.05362601902173836</v>
       </c>
     </row>
     <row r="16">
@@ -2119,23 +2311,23 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cooling_3</t>
+          <t>cooling_1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.7674139492753618</v>
+        <v>0.7528021364795947</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.7021710824275367</v>
+        <v>-0.6453364158163239</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.104769587862318</v>
+        <v>-0.4081911670918323</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.7996150362318843</v>
+        <v>-0.1532884247448933</v>
       </c>
       <c r="G16" t="n">
-        <v>0.8391417572463773</v>
+        <v>0.4540138711734727</v>
       </c>
     </row>
     <row r="17">
@@ -2146,23 +2338,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>cooling_4</t>
+          <t>cooling_2</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.7560320425724605</v>
+        <v>0.9842759284420275</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.6118631114130437</v>
+        <v>-0.8306442481884062</v>
       </c>
       <c r="E17" t="n">
-        <v>0.07668421648550705</v>
+        <v>-0.1593636775362341</v>
       </c>
       <c r="F17" t="n">
-        <v>-1.061280004528989</v>
+        <v>-0.7778391077898554</v>
       </c>
       <c r="G17" t="n">
-        <v>0.8404268568840578</v>
+        <v>0.7835711050724647</v>
       </c>
     </row>
     <row r="18">
@@ -2173,23 +2365,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>demoulding</t>
+          <t>cooling_3</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.8833007812500018</v>
+        <v>0.7674139492753618</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.2243381076388875</v>
+        <v>-0.7021710824275367</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.3624403211805536</v>
+        <v>-0.104769587862318</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.4750162760416643</v>
+        <v>-0.7996150362318843</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1784939236111125</v>
+        <v>0.8391417572463773</v>
       </c>
     </row>
     <row r="19">
@@ -2200,23 +2392,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>deposition_transfer</t>
+          <t>cooling_4</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.2731445312499936</v>
+        <v>0.7560320425724605</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.6679492187500067</v>
+        <v>-0.6118631114130437</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1541601562500041</v>
+        <v>0.07668421648550705</v>
       </c>
       <c r="F19" t="n">
-        <v>0.5771093749999956</v>
+        <v>-1.061280004528989</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.02814453125000682</v>
+        <v>0.8404268568840578</v>
       </c>
     </row>
     <row r="20">
@@ -2227,23 +2419,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>less_periodic_cooling_2</t>
+          <t>demoulding_twisting</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.9534987541528235</v>
+        <v>0.9197916666666686</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.3407223318106318</v>
+        <v>-0.2332031249999993</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0008506800249161728</v>
+        <v>-0.3393229166666654</v>
       </c>
       <c r="F20" t="n">
-        <v>-1.057600316652824</v>
+        <v>-0.5359374999999993</v>
       </c>
       <c r="G20" t="n">
-        <v>0.4439732142857142</v>
+        <v>0.1886718750000007</v>
       </c>
     </row>
     <row r="21">
@@ -2254,23 +2446,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>mould_conditioning</t>
+          <t>demoulding_vibration</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.1637898763020829</v>
+        <v>0.8861799568965516</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.4071329752604171</v>
+        <v>-0.2240369073275872</v>
       </c>
       <c r="E21" t="n">
-        <v>0.06388549804687571</v>
+        <v>-0.3640894396551726</v>
       </c>
       <c r="F21" t="n">
-        <v>0.1546447753906257</v>
+        <v>-0.4750808189655178</v>
       </c>
       <c r="G21" t="n">
-        <v>0.02481282552083286</v>
+        <v>0.1770272090517224</v>
       </c>
     </row>
     <row r="22">
@@ -2281,23 +2473,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>movement_to_conditioning</t>
+          <t>deposition_transfer</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.5641601562500007</v>
+        <v>0.2731445312499936</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.008886718750000355</v>
+        <v>-0.6679492187500067</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.2385742187499993</v>
+        <v>-0.1541601562500041</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.31005859375</v>
+        <v>0.5771093749999956</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.006640624999999289</v>
+        <v>-0.02814453125000682</v>
       </c>
     </row>
     <row r="23">
@@ -2308,23 +2500,23 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>transition_2</t>
+          <t>final_demoulding</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.8461961699695113</v>
+        <v>0.8350585937500004</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.2345607850609763</v>
+        <v>-0.2198730468749996</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.3444836128048792</v>
+        <v>-0.3678222656249996</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.5456316692073173</v>
+        <v>-0.4288574218749996</v>
       </c>
       <c r="G23" t="n">
-        <v>0.2784798971036579</v>
+        <v>0.1814941406250004</v>
       </c>
     </row>
     <row r="24">
@@ -2335,23 +2527,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>transition_to_cooling</t>
+          <t>less_periodic_cooling_2</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.4313151041666643</v>
+        <v>0.9534987541528235</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.5489908854166679</v>
+        <v>-0.3407223318106318</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.3546781994047628</v>
+        <v>0.0008506800249161728</v>
       </c>
       <c r="F24" t="n">
-        <v>0.3505161830357117</v>
+        <v>-1.057600316652824</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1218377976190474</v>
+        <v>0.4439732142857142</v>
       </c>
     </row>
     <row r="25">
@@ -2362,27 +2554,135 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>mould_conditioning</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.1637898763020829</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.4071329752604171</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.06388549804687571</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.1546447753906257</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.02481282552083286</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>reference_2291-4160</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>movement_to_conditioning</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.5641601562500007</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.008886718750000355</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-0.2385742187499993</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-0.31005859375</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-0.006640624999999289</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>reference_2291-4160</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>transition_2</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.8461961699695113</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.2345607850609763</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-0.3444836128048792</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-0.5456316692073173</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.2784798971036579</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>reference_2291-4160</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>transition_to_cooling</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.4313151041666643</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.5489908854166679</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-0.3546781994047628</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.3505161830357117</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.1218377976190474</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>reference_2291-4160</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>vibration_warming</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C29" t="n">
         <v>0.3380594544491551</v>
       </c>
-      <c r="D25" t="n">
+      <c r="D29" t="n">
         <v>-0.4605534957627064</v>
       </c>
-      <c r="E25" t="n">
+      <c r="E29" t="n">
         <v>-0.3258375264830455</v>
       </c>
-      <c r="F25" t="n">
+      <c r="F29" t="n">
         <v>0.4250893802966154</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G29" t="n">
         <v>0.02324218750000284</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Aasted temperature-corrected US comparison
</commit_message>
<xml_diff>
--- a/outputs/aasted3_run_comparison/summary/aasted3_contour_data.xlsx
+++ b/outputs/aasted3_run_comparison/summary/aasted3_contour_data.xlsx
@@ -432,12 +432,12 @@
   <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
@@ -1195,7 +1195,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1207,43 +1207,43 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E16" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="F16" t="n">
-        <v>30.41959307787037</v>
+        <v>82.7384932434167</v>
       </c>
       <c r="G16" t="n">
-        <v>22.12476325757576</v>
+        <v>10.09435096153846</v>
       </c>
       <c r="H16" t="n">
-        <v>22.38299005681818</v>
+        <v>10.48610276442308</v>
       </c>
       <c r="I16" t="n">
-        <v>21.84537760416667</v>
+        <v>10.38168569711539</v>
       </c>
       <c r="J16" t="n">
-        <v>22.62479285037879</v>
+        <v>10.46762319711539</v>
       </c>
       <c r="K16" t="n">
-        <v>21.78666548295455</v>
+        <v>11.07151442307692</v>
       </c>
       <c r="L16" t="n">
-        <v>22.20513731060606</v>
+        <v>10.32316706730769</v>
       </c>
       <c r="M16" t="n">
-        <v>22.33262310606061</v>
+        <v>12.00615985576923</v>
       </c>
       <c r="N16" t="n">
-        <v>21.66850142045455</v>
+        <v>10.95237379807692</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1252,46 +1252,46 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="D17" t="n">
-        <v>493</v>
+        <v>214</v>
       </c>
       <c r="E17" t="n">
-        <v>426</v>
+        <v>188</v>
       </c>
       <c r="F17" t="n">
-        <v>27.64735353773485</v>
+        <v>51.04738086482475</v>
       </c>
       <c r="G17" t="n">
-        <v>22.32362272593897</v>
+        <v>15.30934175531915</v>
       </c>
       <c r="H17" t="n">
-        <v>22.73446669600939</v>
+        <v>15.49720536901596</v>
       </c>
       <c r="I17" t="n">
-        <v>22.15354955252348</v>
+        <v>16.1718438331117</v>
       </c>
       <c r="J17" t="n">
-        <v>22.69943423562206</v>
+        <v>16.4478162400266</v>
       </c>
       <c r="K17" t="n">
-        <v>22.3557851012324</v>
+        <v>16.16723113364362</v>
       </c>
       <c r="L17" t="n">
-        <v>22.33242095803991</v>
+        <v>15.76991564162234</v>
       </c>
       <c r="M17" t="n">
-        <v>23.21314278902582</v>
+        <v>21.44313081781915</v>
       </c>
       <c r="N17" t="n">
-        <v>22.36638057511737</v>
+        <v>17.13998088430851</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1300,46 +1300,46 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>493</v>
+        <v>214</v>
       </c>
       <c r="D18" t="n">
-        <v>600</v>
+        <v>315</v>
       </c>
       <c r="E18" t="n">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F18" t="n">
-        <v>18.40996017253675</v>
+        <v>26.83160178829166</v>
       </c>
       <c r="G18" t="n">
-        <v>27.84138093171296</v>
+        <v>26.42771484375</v>
       </c>
       <c r="H18" t="n">
-        <v>28.89122178819444</v>
+        <v>25.7880859375</v>
       </c>
       <c r="I18" t="n">
-        <v>28.3255931712963</v>
+        <v>26.453671875</v>
       </c>
       <c r="J18" t="n">
-        <v>28.19858579282407</v>
+        <v>27.3671484375</v>
       </c>
       <c r="K18" t="n">
-        <v>28.04537398726852</v>
+        <v>26.76517578125</v>
       </c>
       <c r="L18" t="n">
-        <v>27.98318142361111</v>
+        <v>26.292109375</v>
       </c>
       <c r="M18" t="n">
-        <v>28.87076822916667</v>
+        <v>28.8582421875</v>
       </c>
       <c r="N18" t="n">
-        <v>27.83769169560185</v>
+        <v>26.9780078125</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1348,46 +1348,46 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>600</v>
+        <v>315</v>
       </c>
       <c r="D19" t="n">
-        <v>646</v>
+        <v>374</v>
       </c>
       <c r="E19" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="F19" t="n">
-        <v>20.08367390689834</v>
+        <v>29.07200360891606</v>
       </c>
       <c r="G19" t="n">
-        <v>28.08763586956522</v>
+        <v>27.13792317708333</v>
       </c>
       <c r="H19" t="n">
-        <v>28.41015625</v>
+        <v>26.51373697916667</v>
       </c>
       <c r="I19" t="n">
-        <v>28.33793308423913</v>
+        <v>26.91458333333333</v>
       </c>
       <c r="J19" t="n">
-        <v>27.99660326086957</v>
+        <v>27.64466145833333</v>
       </c>
       <c r="K19" t="n">
-        <v>27.96586277173913</v>
+        <v>27.44684244791667</v>
       </c>
       <c r="L19" t="n">
-        <v>28.1410495923913</v>
+        <v>27.09723307291667</v>
       </c>
       <c r="M19" t="n">
-        <v>27.27381963315218</v>
+        <v>26.18961588541667</v>
       </c>
       <c r="N19" t="n">
-        <v>27.521484375</v>
+        <v>27.11832682291667</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1396,46 +1396,46 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>646</v>
+        <v>374</v>
       </c>
       <c r="D20" t="n">
-        <v>794</v>
+        <v>519</v>
       </c>
       <c r="E20" t="n">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F20" t="n">
-        <v>22.5690515473382</v>
+        <v>29.47016381341881</v>
       </c>
       <c r="G20" t="n">
-        <v>27.60821322737069</v>
+        <v>26.97638617621528</v>
       </c>
       <c r="H20" t="n">
-        <v>27.67869410021552</v>
+        <v>26.18088107638889</v>
       </c>
       <c r="I20" t="n">
-        <v>27.77015422952586</v>
+        <v>26.42420789930556</v>
       </c>
       <c r="J20" t="n">
-        <v>27.29754849137931</v>
+        <v>27.11028374565972</v>
       </c>
       <c r="K20" t="n">
-        <v>27.37843480603448</v>
+        <v>27.03420681423611</v>
       </c>
       <c r="L20" t="n">
-        <v>27.43121969288793</v>
+        <v>26.73326280381944</v>
       </c>
       <c r="M20" t="n">
-        <v>24.94090113146552</v>
+        <v>24.54667154947917</v>
       </c>
       <c r="N20" t="n">
-        <v>26.74345029633621</v>
+        <v>26.47709147135417</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1444,46 +1444,46 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>794</v>
+        <v>519</v>
       </c>
       <c r="D21" t="n">
-        <v>891</v>
+        <v>617</v>
       </c>
       <c r="E21" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F21" t="n">
-        <v>31.26008628754608</v>
+        <v>32.64448837815632</v>
       </c>
       <c r="G21" t="n">
-        <v>26.036865234375</v>
+        <v>25.35172193877551</v>
       </c>
       <c r="H21" t="n">
-        <v>25.24886067708333</v>
+        <v>23.9987643494898</v>
       </c>
       <c r="I21" t="n">
-        <v>25.42427571614583</v>
+        <v>24.32790577168367</v>
       </c>
       <c r="J21" t="n">
-        <v>25.34897867838542</v>
+        <v>24.44174505739796</v>
       </c>
       <c r="K21" t="n">
-        <v>24.54620361328125</v>
+        <v>23.84375</v>
       </c>
       <c r="L21" t="n">
-        <v>25.5823974609375</v>
+        <v>24.99988042091837</v>
       </c>
       <c r="M21" t="n">
-        <v>19.31650797526042</v>
+        <v>18.33225047831633</v>
       </c>
       <c r="N21" t="n">
-        <v>23.711181640625</v>
+        <v>22.97678172831633</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1492,46 +1492,46 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>891</v>
+        <v>617</v>
       </c>
       <c r="D22" t="n">
-        <v>1040</v>
+        <v>793</v>
       </c>
       <c r="E22" t="n">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="F22" t="n">
-        <v>43.80239717798488</v>
+        <v>41.5088553663702</v>
       </c>
       <c r="G22" t="n">
-        <v>22.29559491131757</v>
+        <v>21.95192649147727</v>
       </c>
       <c r="H22" t="n">
-        <v>21.28576330236486</v>
+        <v>20.27727716619318</v>
       </c>
       <c r="I22" t="n">
-        <v>20.90987911739865</v>
+        <v>20.95330255681818</v>
       </c>
       <c r="J22" t="n">
-        <v>22.23527238175676</v>
+        <v>20.3026123046875</v>
       </c>
       <c r="K22" t="n">
-        <v>19.58548880912162</v>
+        <v>19.373291015625</v>
       </c>
       <c r="L22" t="n">
-        <v>21.83449904983108</v>
+        <v>21.778076171875</v>
       </c>
       <c r="M22" t="n">
-        <v>14.56046769425676</v>
+        <v>15.17110928622159</v>
       </c>
       <c r="N22" t="n">
-        <v>19.36277977195946</v>
+        <v>18.49111106178977</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1540,46 +1540,46 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1040</v>
+        <v>793</v>
       </c>
       <c r="D23" t="n">
-        <v>1152</v>
+        <v>900</v>
       </c>
       <c r="E23" t="n">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="F23" t="n">
-        <v>46.59697963747105</v>
+        <v>49.8847423508812</v>
       </c>
       <c r="G23" t="n">
-        <v>19.89169034090909</v>
+        <v>19.87210648148148</v>
       </c>
       <c r="H23" t="n">
-        <v>18.7251953125</v>
+        <v>18.44093605324074</v>
       </c>
       <c r="I23" t="n">
-        <v>18.09115767045455</v>
+        <v>19.13789424189815</v>
       </c>
       <c r="J23" t="n">
-        <v>20.30078125</v>
+        <v>18.49580439814815</v>
       </c>
       <c r="K23" t="n">
-        <v>17.33510298295455</v>
+        <v>16.8963939525463</v>
       </c>
       <c r="L23" t="n">
-        <v>19.80079900568182</v>
+        <v>19.98220486111111</v>
       </c>
       <c r="M23" t="n">
-        <v>14.14669744318182</v>
+        <v>13.9725658275463</v>
       </c>
       <c r="N23" t="n">
-        <v>17.10118963068182</v>
+        <v>16.11273871527778</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1588,46 +1588,46 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1152</v>
+        <v>900</v>
       </c>
       <c r="D24" t="n">
-        <v>1307</v>
+        <v>1024</v>
       </c>
       <c r="E24" t="n">
-        <v>155</v>
+        <v>124</v>
       </c>
       <c r="F24" t="n">
-        <v>49.02330759342392</v>
+        <v>53.36382353946786</v>
       </c>
       <c r="G24" t="n">
-        <v>19.14593184621711</v>
+        <v>19.67872668850806</v>
       </c>
       <c r="H24" t="n">
-        <v>17.85641961348684</v>
+        <v>18.35751638104839</v>
       </c>
       <c r="I24" t="n">
-        <v>17.23269171463816</v>
+        <v>18.98243762600806</v>
       </c>
       <c r="J24" t="n">
-        <v>19.48482473273026</v>
+        <v>18.22352255544355</v>
       </c>
       <c r="K24" t="n">
-        <v>16.58528217516447</v>
+        <v>16.86742376512097</v>
       </c>
       <c r="L24" t="n">
-        <v>19.27977230674342</v>
+        <v>19.84611265120968</v>
       </c>
       <c r="M24" t="n">
-        <v>13.66275185032895</v>
+        <v>14.60827242943548</v>
       </c>
       <c r="N24" t="n">
-        <v>16.06689453125</v>
+        <v>16.29996219758064</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1636,46 +1636,46 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1307</v>
+        <v>1024</v>
       </c>
       <c r="D25" t="n">
-        <v>2035</v>
+        <v>1976</v>
       </c>
       <c r="E25" t="n">
-        <v>728</v>
+        <v>952</v>
       </c>
       <c r="F25" t="n">
-        <v>49.96856924279216</v>
+        <v>58.53781827523181</v>
       </c>
       <c r="G25" t="n">
-        <v>16.77396771121884</v>
+        <v>16.41107741924895</v>
       </c>
       <c r="H25" t="n">
-        <v>14.41952692174515</v>
+        <v>15.19958803834034</v>
       </c>
       <c r="I25" t="n">
-        <v>14.14381979310942</v>
+        <v>15.45544331013656</v>
       </c>
       <c r="J25" t="n">
-        <v>15.66035102146814</v>
+        <v>14.73225979845063</v>
       </c>
       <c r="K25" t="n">
-        <v>14.12902798216759</v>
+        <v>13.97331891741071</v>
       </c>
       <c r="L25" t="n">
-        <v>16.64899746797091</v>
+        <v>15.9488863904937</v>
       </c>
       <c r="M25" t="n">
-        <v>12.36247781769391</v>
+        <v>12.03108176864496</v>
       </c>
       <c r="N25" t="n">
-        <v>13.34616570723684</v>
+        <v>13.81085051207983</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1684,46 +1684,46 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2035</v>
+        <v>1976</v>
       </c>
       <c r="D26" t="n">
-        <v>2074</v>
+        <v>2118</v>
       </c>
       <c r="E26" t="n">
-        <v>39</v>
+        <v>142</v>
       </c>
       <c r="F26" t="n">
-        <v>47.81232937856691</v>
+        <v>64.47090038593441</v>
       </c>
       <c r="G26" t="n">
-        <v>15.203125</v>
+        <v>14.01825209066901</v>
       </c>
       <c r="H26" t="n">
-        <v>13.226953125</v>
+        <v>13.26171875</v>
       </c>
       <c r="I26" t="n">
-        <v>13.240234375</v>
+        <v>12.93784386003521</v>
       </c>
       <c r="J26" t="n">
-        <v>13.610302734375</v>
+        <v>12.95212092869718</v>
       </c>
       <c r="K26" t="n">
-        <v>13.287548828125</v>
+        <v>12.46539392605634</v>
       </c>
       <c r="L26" t="n">
-        <v>14.919091796875</v>
+        <v>13.4679384903169</v>
       </c>
       <c r="M26" t="n">
-        <v>13.68056640625</v>
+        <v>13.57427376760563</v>
       </c>
       <c r="N26" t="n">
-        <v>12.71396484375</v>
+        <v>12.70447293133803</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1732,46 +1732,46 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2074</v>
+        <v>2118</v>
       </c>
       <c r="D27" t="n">
-        <v>2081</v>
+        <v>2126</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F27" t="n">
-        <v>45.34554205390111</v>
+        <v>66.56376596050438</v>
       </c>
       <c r="G27" t="n">
-        <v>15.365234375</v>
+        <v>14.614990234375</v>
       </c>
       <c r="H27" t="n">
-        <v>13.4091796875</v>
+        <v>13.8203125</v>
       </c>
       <c r="I27" t="n">
-        <v>13.37890625</v>
+        <v>13.5830078125</v>
       </c>
       <c r="J27" t="n">
-        <v>13.83072916666667</v>
+        <v>13.44921875</v>
       </c>
       <c r="K27" t="n">
-        <v>13.61165364583333</v>
+        <v>13.414306640625</v>
       </c>
       <c r="L27" t="n">
-        <v>15.05859375</v>
+        <v>13.9560546875</v>
       </c>
       <c r="M27" t="n">
-        <v>14.35286458333333</v>
+        <v>14.666015625</v>
       </c>
       <c r="N27" t="n">
-        <v>13.24251302083333</v>
+        <v>13.785400390625</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1780,46 +1780,46 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2081</v>
+        <v>2126</v>
       </c>
       <c r="D28" t="n">
-        <v>2137</v>
+        <v>2190</v>
       </c>
       <c r="E28" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="F28" t="n">
-        <v>-4.087239910377834</v>
+        <v>65.86329101086693</v>
       </c>
       <c r="G28" t="n">
-        <v>2.28443287037037</v>
+        <v>14.8212890625</v>
       </c>
       <c r="H28" t="n">
-        <v>1.99609375</v>
+        <v>14.09332682291667</v>
       </c>
       <c r="I28" t="n">
-        <v>1.990668402777778</v>
+        <v>13.87932942708333</v>
       </c>
       <c r="J28" t="n">
-        <v>2.058702256944445</v>
+        <v>13.75045572916667</v>
       </c>
       <c r="K28" t="n">
-        <v>2.03833912037037</v>
+        <v>13.93385416666667</v>
       </c>
       <c r="L28" t="n">
-        <v>2.237232349537037</v>
+        <v>14.23974609375</v>
       </c>
       <c r="M28" t="n">
-        <v>2.177734375</v>
+        <v>15.14537760416667</v>
       </c>
       <c r="N28" t="n">
-        <v>1.976345486111111</v>
+        <v>14.16178385416667</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1828,40 +1828,40 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2137</v>
+        <v>2190</v>
       </c>
       <c r="D29" t="n">
-        <v>2141</v>
+        <v>2214</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="F29" t="n">
-        <v>-12.5</v>
+        <v>64.89283327573243</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>15.046875</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>14.37972005208333</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>14.16609700520833</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>14.08349609375</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>14.4072265625</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>14.54166666666667</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>15.45426432291667</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>14.632568359375</v>
       </c>
     </row>
   </sheetData>
@@ -1879,12 +1879,12 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1928,7 +1928,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1937,25 +1937,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.5085896809895836</v>
+        <v>0.7277184311224509</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.2794148763020843</v>
+        <v>-0.6252391581632644</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.1039998372395843</v>
+        <v>-0.2960977359693864</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.1792968749999986</v>
+        <v>-0.1822584502551017</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05412190755208357</v>
+        <v>0.375876913265305</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1964,25 +1964,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5833931587837853</v>
+        <v>0.8992875532670439</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.42643845016892</v>
+        <v>-0.775361772017046</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.802322635135134</v>
+        <v>-0.09933638139204604</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5230706292229748</v>
+        <v>-0.7500266335227295</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1222972972972975</v>
+        <v>0.7254372336647705</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1991,25 +1991,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.5297656249999996</v>
+        <v>0.686317274305555</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.6367294034090918</v>
+        <v>-0.7448531539351855</v>
       </c>
       <c r="E4" t="n">
-        <v>-1.270767045454544</v>
+        <v>-0.04789496527777715</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9388565340909096</v>
+        <v>-0.6899848090277771</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4388742897727269</v>
+        <v>0.7964156539351848</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2018,25 +2018,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.5460038034539458</v>
+        <v>0.6610635080645153</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.7435084292763179</v>
+        <v>-0.6601467993951609</v>
       </c>
       <c r="E5" t="n">
-        <v>-1.367236328125003</v>
+        <v>-0.0352255544354847</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8848966899671034</v>
+        <v>-0.7941406250000007</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6798442639802609</v>
+        <v>0.8284494707661274</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2045,25 +2045,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.156705729166669</v>
+        <v>0.7302734374999993</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.7993489583333311</v>
+        <v>-0.06440429687500071</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.8296223958333311</v>
+        <v>-0.3017089843750007</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.377799479166665</v>
+        <v>-0.4354980468750007</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8500651041666689</v>
+        <v>0.07133789062499929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2072,25 +2072,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.1710069444444442</v>
+        <v>0.6644596354166659</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.117332175925926</v>
+        <v>-0.06350260416666664</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1227575231481484</v>
+        <v>-0.2775000000000016</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0547236689814814</v>
+        <v>-0.406373697916667</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1238064236111112</v>
+        <v>0.08291666666666586</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2099,25 +2099,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-0.4066116898148167</v>
+        <v>-0.03803124999999952</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6432291666666643</v>
+        <v>-0.6776601562499991</v>
       </c>
       <c r="E8" t="n">
-        <v>0.07760054976851904</v>
+        <v>-0.01207421874999781</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.04940682870370594</v>
+        <v>0.9014023437500001</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.2648111979166679</v>
+        <v>-0.1736367187500001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2126,25 +2126,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.6033040364583311</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>-0.06385091145833499</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>-0.277473958333335</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>-0.3600748697916689</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>0.09809570312499716</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2153,25 +2153,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.244635128116345</v>
+        <v>0.8616264279149188</v>
       </c>
       <c r="D10" t="n">
-        <v>-1.10980566135734</v>
+        <v>-0.3498629529936963</v>
       </c>
       <c r="E10" t="n">
-        <v>-1.385512789993074</v>
+        <v>-0.0940076811974766</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1310184383656505</v>
+        <v>-0.817191192883401</v>
       </c>
       <c r="G10" t="n">
-        <v>1.119664884868422</v>
+        <v>0.3994353991596657</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2180,25 +2180,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.1250761076877893</v>
+        <v>-0.5298828125000004</v>
       </c>
       <c r="D11" t="n">
-        <v>0.285767862382631</v>
+        <v>-0.3420191988031931</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.2951492811032814</v>
+        <v>0.3326192652925517</v>
       </c>
       <c r="F11" t="n">
-        <v>0.250735401995307</v>
+        <v>0.6085916722074476</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1162778755868494</v>
+        <v>-0.0693089261968094</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2207,25 +2207,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.1118489583333364</v>
+        <v>-0.2562349759615401</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1463778409090892</v>
+        <v>0.1355168269230749</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.3912346117424264</v>
+        <v>0.03109975961538325</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3881806344696948</v>
+        <v>0.1170372596153832</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.03147490530303187</v>
+        <v>-0.02741887019231015</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2234,25 +2234,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.16318359375</v>
+        <v>0.6906772667253538</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.81298828125</v>
+        <v>-0.06585607394366022</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.7997070312499996</v>
+        <v>-0.3897309639084483</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.4296386718749989</v>
+        <v>-0.3754538952464763</v>
       </c>
       <c r="G13" t="n">
-        <v>0.879150390625</v>
+        <v>0.1403636663732417</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2261,25 +2261,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.05104727909483131</v>
+        <v>0.2913818359374964</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1215281519396569</v>
+        <v>-0.5041232638888928</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2129882812500021</v>
+        <v>-0.260796440972225</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2596174568965495</v>
+        <v>0.4252794053819393</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.1259462553879267</v>
+        <v>0.04825846354166075</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>old-configuration</t>
+          <t>17_3_f_m_aa3-25_06_26-2160-4374s</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2288,19 +2288,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-0.1070397418478244</v>
+        <v>0.076295572916667</v>
       </c>
       <c r="D15" t="n">
-        <v>0.215480638586957</v>
+        <v>-0.5478906250000009</v>
       </c>
       <c r="E15" t="n">
-        <v>0.143257472826086</v>
+        <v>-0.1470442708333337</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.1980723505434767</v>
+        <v>0.5830338541666684</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.05362601902173836</v>
+        <v>0.03560546874999915</v>
       </c>
     </row>
     <row r="16">

</xml_diff>